<commit_message>
Ajout des KPI, de la table Calendrier et des maquettes HTML
- kpis/ : catalogue de 34 KPI et spécification des pages
  Overview, Clients et Ventes
- Modèle TMDL : table Calendrier (table de dates) reliée aux ventes,
  34 mesures rangées par dossier (Ventes, Temps, Remises, Clients)
- Jeu de données plus réaliste : noms de clients uniques, arrivées et
  départs de clients, saisonnalité ; fichiers Excel reproductibles
- ui/ : maquettes HTML des 3 pages avec filtres partagés, KPI calculés
  comme les mesures DAX et graphiques SVG sans dépendance

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/sources/Clients.xlsx
+++ b/sources/Clients.xlsx
@@ -495,12 +495,12 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>Studio Durand</t>
+          <t>Rousseau Dubois</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
@@ -510,7 +510,7 @@
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -520,22 +520,22 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Rousseau Dubois</t>
+          <t>Groupe Simon</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -545,22 +545,22 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Atelier Dubois</t>
+          <t>Rousseau Bonnet</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -570,17 +570,17 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Maison Martin</t>
+          <t>Comptoir Martin</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -595,22 +595,22 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Studio Rousseau</t>
+          <t>Roux Michel</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -620,22 +620,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Maison Michel</t>
+          <t>Atelier Fournier</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -645,22 +645,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Moreau Bonnet</t>
+          <t>Atelier Dupont</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -670,22 +670,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Groupe Roux</t>
+          <t>Société Muller</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -695,22 +695,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>Atelier Fournier</t>
+          <t>Dubois Bernard</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -720,22 +720,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>Bernard Dupont</t>
+          <t>Atelier Simon</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -745,22 +745,22 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>Cabinet Dubois</t>
+          <t>Studio Fournier</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -770,22 +770,22 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Studio Muller</t>
+          <t>Dubois Muller</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -795,17 +795,17 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Dubois Bernard</t>
+          <t>Moreau Dupont</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Nouvelle-Aquitaine</t>
         </is>
       </c>
       <c r="E15" t="inlineStr">
@@ -820,7 +820,7 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>Société Dubois</t>
+          <t>Simon Roux</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
@@ -835,7 +835,7 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -845,22 +845,22 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Girard Michel</t>
+          <t>Comptoir Bernard</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -870,17 +870,17 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>Fournier Moreau</t>
+          <t>Vincent Roux</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -895,17 +895,17 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>Studio Michel</t>
+          <t>Société Lefebvre</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
@@ -920,7 +920,7 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>Dubois Muller</t>
+          <t>Vincent Girard</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
@@ -945,22 +945,22 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>Studio Simon</t>
+          <t>Durand Lefebvre</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -970,17 +970,17 @@
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>Société Rousseau</t>
+          <t>Cabinet Fontaine</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E22" t="inlineStr">
@@ -995,17 +995,17 @@
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>Bernard Simon</t>
+          <t>Durand Rousseau</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
@@ -1020,22 +1020,22 @@
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>Girard Michel</t>
+          <t>Maison Moreau</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1045,22 +1045,22 @@
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>Maison Roux</t>
+          <t>Fontaine Muller</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1070,17 +1070,17 @@
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>Girard Dupont</t>
+          <t>Fontaine Martin</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D26" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Nouvelle-Aquitaine</t>
         </is>
       </c>
       <c r="E26" t="inlineStr">
@@ -1095,17 +1095,17 @@
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>Groupe Rousseau</t>
+          <t>Maison Dubois</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E27" t="inlineStr">
@@ -1120,22 +1120,22 @@
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>Maison Bonnet</t>
+          <t>Lefebvre Lefebvre</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D28" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1145,22 +1145,22 @@
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>Groupe Lefebvre</t>
+          <t>Laurent Garcia</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D29" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1170,22 +1170,22 @@
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>Comptoir Bernard</t>
+          <t>Dupont Durand</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1195,22 +1195,22 @@
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>Groupe Bonnet</t>
+          <t>Vincent Simon</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1220,17 +1220,17 @@
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>Cabinet Muller</t>
+          <t>Atelier Roux</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E32" t="inlineStr">
@@ -1245,7 +1245,7 @@
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Rousseau Martin</t>
+          <t>Groupe Vincent</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -1260,7 +1260,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1270,22 +1270,22 @@
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Rousseau Michel</t>
+          <t>Atelier Durand</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1295,17 +1295,17 @@
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Durand Garcia</t>
+          <t>Bernard Durand</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E35" t="inlineStr">
@@ -1320,17 +1320,17 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Atelier Michel</t>
+          <t>Groupe Rousseau</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E36" t="inlineStr">
@@ -1345,17 +1345,17 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Fontaine Durand</t>
+          <t>Dubois Dupont</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E37" t="inlineStr">
@@ -1370,22 +1370,22 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>Studio Fontaine</t>
+          <t>Simon Moreau</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1395,22 +1395,22 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>Société Moreau</t>
+          <t>Moreau Girard</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D39" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1420,17 +1420,17 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Fontaine Martin</t>
+          <t>Garcia Bonnet</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D40" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E40" t="inlineStr">
@@ -1445,17 +1445,17 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Atelier Durand</t>
+          <t>Société Laurent</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D41" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E41" t="inlineStr">
@@ -1470,22 +1470,22 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Garcia Simon</t>
+          <t>Comptoir Fontaine</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E42" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -1495,12 +1495,12 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Maison Dubois</t>
+          <t>Simon Girard</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
@@ -1510,7 +1510,7 @@
       </c>
       <c r="E43" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1520,22 +1520,22 @@
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Dubois Rousseau</t>
+          <t>Atelier Bonnet</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E44" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -1545,17 +1545,17 @@
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Studio Lambert</t>
+          <t>Studio Roux</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E45" t="inlineStr">
@@ -1570,17 +1570,17 @@
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Maison Muller</t>
+          <t>Comptoir Dubois</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E46" t="inlineStr">
@@ -1595,22 +1595,22 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Rousseau Laurent</t>
+          <t>Groupe Fontaine</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E47" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -1620,17 +1620,17 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Studio Fournier</t>
+          <t>Groupe Dupont</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>Grand Est</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E48" t="inlineStr">
@@ -1645,17 +1645,17 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Dupont Durand</t>
+          <t>Martin Rousseau</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E49" t="inlineStr">
@@ -1670,22 +1670,22 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Société Martin</t>
+          <t>Atelier Rousseau</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E50" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -1695,22 +1695,22 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Vincent Simon</t>
+          <t>Maison Lambert</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E51" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1720,17 +1720,17 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Studio Bernard</t>
+          <t>Maison Bonnet</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E52" t="inlineStr">
@@ -1745,12 +1745,12 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Atelier Roux</t>
+          <t>Fournier Vincent</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
@@ -1760,7 +1760,7 @@
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1770,17 +1770,17 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Michel Lambert</t>
+          <t>Bernard Fournier</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E54" t="inlineStr">
@@ -1795,17 +1795,17 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Vincent Vincent</t>
+          <t>Bonnet Muller</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Nice</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E55" t="inlineStr">
@@ -1820,22 +1820,22 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Cabinet Bonnet</t>
+          <t>Bonnet Martin</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1845,22 +1845,22 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Studio Bonnet</t>
+          <t>Simon Michel</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1870,17 +1870,17 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Cabinet Bernard</t>
+          <t>Comptoir Dupont</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E58" t="inlineStr">
@@ -1895,7 +1895,7 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Durand Bernard</t>
+          <t>Société Michel</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -1910,7 +1910,7 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1920,22 +1920,22 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Durand Simon</t>
+          <t>Comptoir Rousseau</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Nouvelle-Aquitaine</t>
         </is>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -1945,12 +1945,12 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Cabinet Lefebvre</t>
+          <t>Michel Bernard</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
@@ -1960,7 +1960,7 @@
       </c>
       <c r="E61" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -1970,17 +1970,17 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Cabinet Simon</t>
+          <t>Maison Fontaine</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E62" t="inlineStr">
@@ -1995,17 +1995,17 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Comptoir Rousseau</t>
+          <t>Maison Rousseau</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E63" t="inlineStr">
@@ -2020,7 +2020,7 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Maison Martin</t>
+          <t>Roux Muller</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
@@ -2035,7 +2035,7 @@
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2045,17 +2045,17 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Simon Moreau</t>
+          <t>Bonnet Roux</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E65" t="inlineStr">
@@ -2070,17 +2070,17 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Groupe Girard</t>
+          <t>Cabinet Moreau</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E66" t="inlineStr">
@@ -2095,7 +2095,7 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Atelier Girard</t>
+          <t>Groupe Bonnet</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
@@ -2120,17 +2120,17 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Dupont Garcia</t>
+          <t>Fontaine Lambert</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E68" t="inlineStr">
@@ -2145,17 +2145,17 @@
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Rousseau Lambert</t>
+          <t>Muller Roux</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Marseille</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Provence-Alpes-Côte d'Azur</t>
         </is>
       </c>
       <c r="E69" t="inlineStr">
@@ -2170,12 +2170,12 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Groupe Bernard</t>
+          <t>Lefebvre Martin</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
@@ -2185,7 +2185,7 @@
       </c>
       <c r="E70" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2195,22 +2195,22 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Bernard Roux</t>
+          <t>Cabinet Vincent</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -2220,22 +2220,22 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Cabinet Fontaine</t>
+          <t>Studio Martin</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2245,17 +2245,17 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Maison Dubois</t>
+          <t>Studio Fontaine</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E73" t="inlineStr">
@@ -2270,22 +2270,22 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Atelier Simon</t>
+          <t>Maison Muller</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2295,22 +2295,22 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Maison Simon</t>
+          <t>Bonnet Rousseau</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E75" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2320,22 +2320,22 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Muller Dubois</t>
+          <t>Comptoir Simon</t>
         </is>
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>Nantes</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>Pays de la Loire</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E76" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2345,22 +2345,22 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Vincent Fontaine</t>
+          <t>Groupe Michel</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Bordeaux</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Nouvelle-Aquitaine</t>
         </is>
       </c>
       <c r="E77" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2370,7 +2370,7 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Laurent Roux</t>
+          <t>Groupe Lefebvre</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -2385,7 +2385,7 @@
       </c>
       <c r="E78" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2395,17 +2395,17 @@
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>Groupe Garcia</t>
+          <t>Société Rousseau</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
@@ -2420,12 +2420,12 @@
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>Comptoir Dubois</t>
+          <t>Comptoir Vincent</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
@@ -2445,22 +2445,22 @@
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>Maison Durand</t>
+          <t>Lambert Martin</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E81" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2470,17 +2470,17 @@
       </c>
       <c r="B82" t="inlineStr">
         <is>
-          <t>Fontaine Michel</t>
+          <t>Rousseau Muller</t>
         </is>
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
@@ -2495,22 +2495,22 @@
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>Dubois Simon</t>
+          <t>Cabinet Roux</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2520,22 +2520,22 @@
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>Cabinet Rousseau</t>
+          <t>Muller Rousseau</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D84" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2545,22 +2545,22 @@
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>Comptoir Fontaine</t>
+          <t>Studio Bonnet</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D85" t="inlineStr">
         <is>
-          <t>Grand Est</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="E85" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -2570,22 +2570,22 @@
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>Rousseau Garcia</t>
+          <t>Société Girard</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D86" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E86" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2595,22 +2595,22 @@
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>Groupe Michel</t>
+          <t>Studio Rousseau</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D87" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E87" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2620,7 +2620,7 @@
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>Rousseau Lefebvre</t>
+          <t>Bernard Martin</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -2645,17 +2645,17 @@
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>Groupe Roux</t>
+          <t>Groupe Lambert</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D89" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E89" t="inlineStr">
@@ -2670,17 +2670,17 @@
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>Michel Fontaine</t>
+          <t>Fournier Moreau</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D90" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E90" t="inlineStr">
@@ -2695,22 +2695,22 @@
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>Comptoir Bernard</t>
+          <t>Durand Vincent</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D91" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E91" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2720,22 +2720,22 @@
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>Michel Bernard</t>
+          <t>Studio Laurent</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Toulouse</t>
         </is>
       </c>
       <c r="D92" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E92" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -2745,22 +2745,22 @@
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>Groupe Michel</t>
+          <t>Comptoir Garcia</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D93" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E93" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -2770,17 +2770,17 @@
       </c>
       <c r="B94" t="inlineStr">
         <is>
-          <t>Rousseau Bonnet</t>
+          <t>Fournier Rousseau</t>
         </is>
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D94" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E94" t="inlineStr">
@@ -2795,22 +2795,22 @@
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>Atelier Lefebvre</t>
+          <t>Lambert Durand</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D95" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E95" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2820,22 +2820,22 @@
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>Société Vincent</t>
+          <t>Bonnet Moreau</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>Bordeaux</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>Nouvelle-Aquitaine</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E96" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2845,7 +2845,7 @@
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>Groupe Bernard</t>
+          <t>Dupont Bonnet</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
@@ -2860,7 +2860,7 @@
       </c>
       <c r="E97" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2870,22 +2870,22 @@
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>Comptoir Bernard</t>
+          <t>Dubois Michel</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>Marseille</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D98" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2895,22 +2895,22 @@
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>Groupe Durand</t>
+          <t>Girard Roux</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D99" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       </c>
       <c r="B100" t="inlineStr">
         <is>
-          <t>Bonnet Muller</t>
+          <t>Muller Michel</t>
         </is>
       </c>
       <c r="C100" t="inlineStr">
@@ -2945,17 +2945,17 @@
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>Groupe Moreau</t>
+          <t>Cabinet Lambert</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>Grand Est</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E101" t="inlineStr">
@@ -2970,17 +2970,17 @@
       </c>
       <c r="B102" t="inlineStr">
         <is>
-          <t>Bonnet Martin</t>
+          <t>Dupont Martin</t>
         </is>
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="E102" t="inlineStr">
@@ -2995,12 +2995,12 @@
       </c>
       <c r="B103" t="inlineStr">
         <is>
-          <t>Roux Bonnet</t>
+          <t>Maison Fournier</t>
         </is>
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
@@ -3010,7 +3010,7 @@
       </c>
       <c r="E103" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3020,17 +3020,17 @@
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>Simon Michel</t>
+          <t>Fournier Dupont</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E104" t="inlineStr">
@@ -3045,22 +3045,22 @@
       </c>
       <c r="B105" t="inlineStr">
         <is>
-          <t>Durand Girard</t>
+          <t>Comptoir Moreau</t>
         </is>
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E105" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3070,17 +3070,17 @@
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>Simon Laurent</t>
+          <t>Garcia Durand</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E106" t="inlineStr">
@@ -3095,17 +3095,17 @@
       </c>
       <c r="B107" t="inlineStr">
         <is>
-          <t>Comptoir Simon</t>
+          <t>Atelier Bernard</t>
         </is>
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>Montpellier</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E107" t="inlineStr">
@@ -3120,22 +3120,22 @@
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>Groupe Girard</t>
+          <t>Maison Garcia</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>Grenoble</t>
+          <t>Rennes</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Bretagne</t>
         </is>
       </c>
       <c r="E108" t="inlineStr">
         <is>
-          <t>Grand compte</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3145,17 +3145,17 @@
       </c>
       <c r="B109" t="inlineStr">
         <is>
-          <t>Atelier Michel</t>
+          <t>Comptoir Lambert</t>
         </is>
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Paris</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E109" t="inlineStr">
@@ -3170,17 +3170,17 @@
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>Girard Rousseau</t>
+          <t>Bernard Lefebvre</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D110" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E110" t="inlineStr">
@@ -3195,17 +3195,17 @@
       </c>
       <c r="B111" t="inlineStr">
         <is>
-          <t>Durand Michel</t>
+          <t>Muller Muller</t>
         </is>
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>Nice</t>
+          <t>Versailles</t>
         </is>
       </c>
       <c r="D111" t="inlineStr">
         <is>
-          <t>Provence-Alpes-Côte d'Azur</t>
+          <t>Île-de-France</t>
         </is>
       </c>
       <c r="E111" t="inlineStr">
@@ -3220,22 +3220,22 @@
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>Michel Bernard</t>
+          <t>Société Vincent</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>Lyon</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D112" t="inlineStr">
         <is>
-          <t>Auvergne-Rhône-Alpes</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E112" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3245,17 +3245,17 @@
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>Fournier Roux</t>
+          <t>Michel Dubois</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>Versailles</t>
+          <t>Grenoble</t>
         </is>
       </c>
       <c r="D113" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E113" t="inlineStr">
@@ -3270,22 +3270,22 @@
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>Fontaine Durand</t>
+          <t>Cabinet Muller</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D114" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E114" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -3295,22 +3295,22 @@
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>Laurent Michel</t>
+          <t>Cabinet Durand</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Strasbourg</t>
         </is>
       </c>
       <c r="D115" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Grand Est</t>
         </is>
       </c>
       <c r="E115" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3320,22 +3320,22 @@
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>Martin Fontaine</t>
+          <t>Groupe Garcia</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>Paris</t>
+          <t>Lyon</t>
         </is>
       </c>
       <c r="D116" t="inlineStr">
         <is>
-          <t>Île-de-France</t>
+          <t>Auvergne-Rhône-Alpes</t>
         </is>
       </c>
       <c r="E116" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>Grand compte</t>
         </is>
       </c>
     </row>
@@ -3345,17 +3345,17 @@
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>Laurent Fournier</t>
+          <t>Girard Michel</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>Rennes</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>Bretagne</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E117" t="inlineStr">
@@ -3370,17 +3370,17 @@
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>Studio Roux</t>
+          <t>Maison Michel</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>Toulouse</t>
+          <t>Nantes</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>Occitanie</t>
+          <t>Pays de la Loire</t>
         </is>
       </c>
       <c r="E118" t="inlineStr">
@@ -3395,7 +3395,7 @@
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>Comptoir Durand</t>
+          <t>Martin Michel</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -3410,7 +3410,7 @@
       </c>
       <c r="E119" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>
@@ -3420,22 +3420,22 @@
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>Fontaine Garcia</t>
+          <t>Société Moreau</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>Strasbourg</t>
+          <t>Lille</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>Grand Est</t>
+          <t>Hauts-de-France</t>
         </is>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>Particulier</t>
+          <t>PME</t>
         </is>
       </c>
     </row>
@@ -3445,22 +3445,22 @@
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>Cabinet Garcia</t>
+          <t>Lambert Fournier</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>Lille</t>
+          <t>Montpellier</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>Hauts-de-France</t>
+          <t>Occitanie</t>
         </is>
       </c>
       <c r="E121" t="inlineStr">
         <is>
-          <t>PME</t>
+          <t>Particulier</t>
         </is>
       </c>
     </row>

</xml_diff>